<commit_message>
Add AQUANUT news, publish Omukoto paper, fix publication order & buttons
</commit_message>
<xml_diff>
--- a/data/cv.xlsx
+++ b/data/cv.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thomas/Library/Mobile Documents/com~apple~CloudDocs/Github/website/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lamy/MySpace/Github/website/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{165EFB00-51CF-3E46-AE8C-608BC3C6BDE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32888C2C-5A9F-C64C-BDB8-23AAFED4D3F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="31900" windowHeight="19120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="44460" windowHeight="25340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="pubs" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="477">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="484">
   <si>
     <t>category</t>
   </si>
@@ -1417,9 +1417,6 @@
     <t>Regional collaboration on nutrient composition and contaminants in aquatic foods, to strengthen food security in Western Indian Ocean communities</t>
   </si>
   <si>
-    <t xml:space="preserve">Accepted in Western Indian Ocean Journal of Marine Science </t>
-  </si>
-  <si>
     <t>An integrative environmental-DNA framework for identifying key species along ecological gradients: combining sparse classification, co-presence network topology, and gene set enrichment on marine fish habitats from New Caledonia</t>
   </si>
   <si>
@@ -1463,6 +1460,30 @@
   </si>
   <si>
     <t>Off Bali, low-cost passive eDNA samplers matched active filtration in detecting pelagic fish at a fish-aggregating device, a practical, transferable tool for monitoring biodiversity in hard-to-reach waters.</t>
+  </si>
+  <si>
+    <t>10.64898/2026.08.28.26361595</t>
+  </si>
+  <si>
+    <t>https://www.medrxiv.org/content/10.64898/2026.08.28.26361595v1</t>
+  </si>
+  <si>
+    <t>Western Indian Ocean Journal of Marine Science</t>
+  </si>
+  <si>
+    <t>25(2), 23–32</t>
+  </si>
+  <si>
+    <t>https://www.ajol.info/index.php/wiojms/article/view/312281</t>
+  </si>
+  <si>
+    <t>-DxkuPiZhfEC</t>
+  </si>
+  <si>
+    <t>0.4314/wiojms.v25i2.3</t>
+  </si>
+  <si>
+    <t>https://www.ajol.info/index.php/wiojms/article/view/312281/316918</t>
   </si>
 </sst>
 </file>
@@ -1567,7 +1588,7 @@
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1830,10 +1851,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="F1" s="7" t="s">
         <v>3</v>
@@ -1925,8 +1946,14 @@
       <c r="L2" s="2" t="s">
         <v>402</v>
       </c>
-    </row>
-    <row r="3" spans="1:26" ht="51" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="N2" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="O2" s="9" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" ht="39" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="2" t="s">
         <v>400</v>
       </c>
@@ -1944,14 +1971,15 @@
         <v>47</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>461</v>
-      </c>
+        <v>402</v>
+      </c>
+      <c r="P3" s="6"/>
     </row>
     <row r="4" spans="1:26" ht="39" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="2" t="s">
@@ -1974,12 +2002,11 @@
         <v>463</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="L4" s="2" t="s">
         <v>402</v>
       </c>
-      <c r="P4" s="6"/>
     </row>
     <row r="5" spans="1:26" ht="39" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="2" t="s">
@@ -1999,7 +2026,7 @@
         <v>45</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>465</v>
@@ -2008,9 +2035,9 @@
         <v>402</v>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="39" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:26" ht="51" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="2" t="s">
-        <v>400</v>
+        <v>22</v>
       </c>
       <c r="B6" s="6" t="b">
         <v>0</v>
@@ -2022,17 +2049,38 @@
         <v>0</v>
       </c>
       <c r="E6" s="6"/>
+      <c r="F6" s="5">
+        <v>46293</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>481</v>
+      </c>
       <c r="H6" s="2">
         <v>44</v>
       </c>
+      <c r="I6" s="2">
+        <v>2026</v>
+      </c>
       <c r="J6" s="2" t="s">
-        <v>467</v>
+        <v>459</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>466</v>
+        <v>460</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>402</v>
+        <v>478</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>479</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="O6" s="9" t="s">
+        <v>480</v>
+      </c>
+      <c r="Q6" s="9" t="s">
+        <v>483</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="39" customHeight="1" x14ac:dyDescent="0.15">
@@ -2081,13 +2129,13 @@
       </c>
       <c r="P7" s="6"/>
       <c r="Q7" s="9" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="U7" s="2" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="Y7" s="2" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="39" customHeight="1" x14ac:dyDescent="0.15">
@@ -2155,10 +2203,10 @@
         <v>0</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="F9" s="5">
         <v>46133</v>
@@ -2211,10 +2259,10 @@
         <v>0</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="F10" s="5">
         <v>46143</v>
@@ -2302,7 +2350,7 @@
         <v>438</v>
       </c>
       <c r="Q11" s="9" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="U11" s="2" t="s">
         <v>439</v>
@@ -4479,7 +4527,11 @@
     <hyperlink ref="Q12" r:id="rId82" xr:uid="{95BA3876-D019-9D47-A736-377F92CA3702}"/>
     <hyperlink ref="Q11" r:id="rId83" xr:uid="{5CB8BC60-7116-584A-B83D-156E386A4677}"/>
     <hyperlink ref="Q7" r:id="rId84" xr:uid="{27712D7F-759E-3544-8CD3-0A01F0797354}"/>
+    <hyperlink ref="O2" r:id="rId85" xr:uid="{5E858ACB-D932-7949-A006-CBE86BC659B7}"/>
+    <hyperlink ref="O6" r:id="rId86" xr:uid="{E0C544FA-A6A3-244B-B437-4F9DDCF9F5A2}"/>
+    <hyperlink ref="Q6" r:id="rId87" xr:uid="{423544E0-DE85-BB4F-8C32-6A8B5F717A72}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>